<commit_message>
rm useless comments e399b1f152a2965ee350b30b04131fc0e760009b
</commit_message>
<xml_diff>
--- a/nr-create-FrPractitionerRole/ig/StructureDefinition-fr-core-practitioner-role.xlsx
+++ b/nr-create-FrPractitionerRole/ig/StructureDefinition-fr-core-practitioner-role.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="343">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-11T16:34:47+00:00</t>
+    <t>2024-06-11T16:42:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -694,289 +694,119 @@
     <t>FiveWs.identifier</t>
   </si>
   <si>
-    <t>PractitionerRole.identifier.id</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.extension</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.use</t>
-  </si>
-  <si>
-    <t>usual | official | temp | secondary | old (If known)</t>
-  </si>
-  <si>
-    <t>The purpose of this identifier.</t>
-  </si>
-  <si>
-    <t>Applications can assume that an identifier is permanent unless it explicitly says that it is temporary.</t>
-  </si>
-  <si>
-    <t>Allows the appropriate identifier for a particular context of use to be selected from among a set of identifiers.</t>
-  </si>
-  <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>Identifies the purpose for this identifier, if known .</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/identifier-use|4.0.1</t>
-  </si>
-  <si>
-    <t>Identifier.use</t>
-  </si>
-  <si>
-    <t>Role.code or implied by context</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.type</t>
+    <t>PractitionerRole.active</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boolean
+</t>
+  </si>
+  <si>
+    <t>Whether this practitioner role record is in active use</t>
+  </si>
+  <si>
+    <t>Whether this practitioner role record is in active use.</t>
+  </si>
+  <si>
+    <t>If this value is false, you may refer to the period to see when the role was in active use. If there is no period specified, no inference can be made about when it was active.</t>
+  </si>
+  <si>
+    <t>Need to be able to mark a practitioner role record as not to be used because it was created in error, or otherwise no longer in active use.</t>
+  </si>
+  <si>
+    <t>This resource is generally assumed to be active if no value is provided for the active element</t>
+  </si>
+  <si>
+    <t>STF-7</t>
+  </si>
+  <si>
+    <t>.statusCode</t>
+  </si>
+  <si>
+    <t>FiveWs.status</t>
+  </si>
+  <si>
+    <t>PractitionerRole.period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period
+</t>
+  </si>
+  <si>
+    <t>The period during which the practitioner is authorized to perform in these role(s)</t>
+  </si>
+  <si>
+    <t>The period during which the person is authorized to act as a practitioner in these role(s) for the organization.</t>
+  </si>
+  <si>
+    <t>A Period specifies a range of time; the context of use will specify whether the entire range applies (e.g. "the patient was an inpatient of the hospital for this time range") or one value from the range applies (e.g. "give to the patient between these two times").
+Period is not used for a duration (a measure of elapsed time). See [Duration](http://hl7.org/fhir/R4/datatypes.html#Duration).</t>
+  </si>
+  <si>
+    <t>Even after the agencies is revoked, the fact that it existed must still be recorded.</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+per-1:If present, start SHALL have a lower value than end {start.hasValue().not() or end.hasValue().not() or (start &lt;= end)}</t>
+  </si>
+  <si>
+    <t>PRD-8/9 / PRA-5.4</t>
+  </si>
+  <si>
+    <t>.performance[@typeCode &lt;= 'PPRF'].ActDefinitionOrEvent.effectiveTime</t>
+  </si>
+  <si>
+    <t>(ServD maps Practitioners and Organizations via another entity, so this concept is not available)</t>
+  </si>
+  <si>
+    <t>FiveWs.done[x]</t>
+  </si>
+  <si>
+    <t>PractitionerRole.practitioner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-practitioner)
+</t>
+  </si>
+  <si>
+    <t>Practitioner that is able to provide the defined services for the organization</t>
+  </si>
+  <si>
+    <t>Practitioner that is able to provide the defined services for the organization.</t>
+  </si>
+  <si>
+    <t>References SHALL be a reference to an actual FHIR resource, and SHALL be resolveable (allowing for access control, temporary unavailability, etc.). Resolution can be either by retrieval from the URL, or, where applicable by resource type, by treating an absolute reference as a canonical URL and looking it up in a local registry/repository.</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+ref-1:SHALL have a contained resource if a local reference is provided {reference.startsWith('#').not() or (reference.substring(1).trace('url') in %rootResource.contained.id.trace('ids'))}</t>
+  </si>
+  <si>
+    <t>.player</t>
+  </si>
+  <si>
+    <t>PractitionerRole.organization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-organization)
+</t>
+  </si>
+  <si>
+    <t>Organization where the roles are available</t>
+  </si>
+  <si>
+    <t>The organization where the Practitioner performs the roles associated.</t>
+  </si>
+  <si>
+    <t>.scoper</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code</t>
   </si>
   <si>
     <t xml:space="preserve">CodeableConcept
 </t>
   </si>
   <si>
-    <t>Description of identifier</t>
-  </si>
-  <si>
-    <t>A coded type for the identifier that can be used to determine which identifier to use for a specific purpose.</t>
-  </si>
-  <si>
-    <t>This element deals only with general categories of identifiers.  It SHOULD not be used for codes that correspond 1..1 with the Identifier.system. Some identifiers may fall into multiple categories due to common usage.   Where the system is known, a type is unnecessary because the type is always part of the system definition. However systems often need to handle identifiers where the system is not known. There is not a 1:1 relationship between type and system, since many different systems have the same type.</t>
-  </si>
-  <si>
-    <t>Allows users to make use of identifiers when the identifier system is not known.</t>
-  </si>
-  <si>
-    <t>A coded type for an identifier that can be used to determine which identifier to use for a specific purpose.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/identifier-type</t>
-  </si>
-  <si>
-    <t>Identifier.type</t>
-  </si>
-  <si>
-    <t>CX.5</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.system</t>
-  </si>
-  <si>
-    <t>The namespace for the identifier value | Namespace du RASS)</t>
-  </si>
-  <si>
-    <t>Establishes the namespace for the value - that is, a URL that describes a set values that are unique.
-Namespace du RASS)</t>
-  </si>
-  <si>
-    <t>Identifier.system is always case sensitive.</t>
-  </si>
-  <si>
-    <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
-  </si>
-  <si>
-    <t>http://www.acme.com/identifiers/patient</t>
-  </si>
-  <si>
-    <t>Identifier.system</t>
-  </si>
-  <si>
-    <t>CX.4 / EI-2-4</t>
-  </si>
-  <si>
-    <t>II.root or Role.id.root</t>
-  </si>
-  <si>
-    <t>./IdentifierType</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.value</t>
-  </si>
-  <si>
-    <t>The value that is unique</t>
-  </si>
-  <si>
-    <t>The portion of the identifier typically relevant to the user and which is unique within the context of the system.</t>
-  </si>
-  <si>
-    <t>If the value is a full URI, then the system SHALL be urn:ietf:rfc:3986.  The value's primary purpose is computational mapping.  As a result, it may be normalized for comparison purposes (e.g. removing non-significant whitespace, dashes, etc.)  A value formatted for human display can be conveyed using the [Rendered Value extension](http://hl7.org/fhir/R4/extension-rendered-value.html). Identifier.value is to be treated as case sensitive unless knowledge of the Identifier.system allows the processer to be confident that non-case-sensitive processing is safe.</t>
-  </si>
-  <si>
-    <t>123456</t>
-  </si>
-  <si>
-    <t>Identifier.value</t>
-  </si>
-  <si>
-    <t>CX.1 / EI.1</t>
-  </si>
-  <si>
-    <t>II.extension or II.root if system indicates OID or GUID (Or Role.id.extension or root)</t>
-  </si>
-  <si>
-    <t>./Value</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.period</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period
-</t>
-  </si>
-  <si>
-    <t>Time period when id is/was valid for use</t>
-  </si>
-  <si>
-    <t>Time period during which identifier is/was valid for use.</t>
-  </si>
-  <si>
-    <t>A Period specifies a range of time; the context of use will specify whether the entire range applies (e.g. "the patient was an inpatient of the hospital for this time range") or one value from the range applies (e.g. "give to the patient between these two times").
-Period is not used for a duration (a measure of elapsed time). See [Duration](http://hl7.org/fhir/R4/datatypes.html#Duration).</t>
-  </si>
-  <si>
-    <t>Identifier.period</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-per-1:If present, start SHALL have a lower value than end {start.hasValue().not() or end.hasValue().not() or (start &lt;= end)}</t>
-  </si>
-  <si>
-    <t>CX.7 + CX.8</t>
-  </si>
-  <si>
-    <t>Role.effectiveTime or implied by context</t>
-  </si>
-  <si>
-    <t>./StartDate and ./EndDate</t>
-  </si>
-  <si>
-    <t>PractitionerRole.identifier.assigner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Organization)
-</t>
-  </si>
-  <si>
-    <t>Organization that issued id (may be just text)</t>
-  </si>
-  <si>
-    <t>Organization that issued/manages the identifier.</t>
-  </si>
-  <si>
-    <t>The Identifier.assigner may omit the .reference element and only contain a .display element reflecting the name or other textual information about the assigning organization.</t>
-  </si>
-  <si>
-    <t>Identifier.assigner</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ref-1:SHALL have a contained resource if a local reference is provided {reference.startsWith('#').not() or (reference.substring(1).trace('url') in %rootResource.contained.id.trace('ids'))}</t>
-  </si>
-  <si>
-    <t>CX.4 / (CX.4,CX.9,CX.10)</t>
-  </si>
-  <si>
-    <t>II.assigningAuthorityName but note that this is an improper use by the definition of the field.  Also Role.scoper</t>
-  </si>
-  <si>
-    <t>./IdentifierIssuingAuthority</t>
-  </si>
-  <si>
-    <t>PractitionerRole.active</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boolean
-</t>
-  </si>
-  <si>
-    <t>Whether this practitioner role record is in active use</t>
-  </si>
-  <si>
-    <t>Whether this practitioner role record is in active use.</t>
-  </si>
-  <si>
-    <t>If this value is false, you may refer to the period to see when the role was in active use. If there is no period specified, no inference can be made about when it was active.</t>
-  </si>
-  <si>
-    <t>Need to be able to mark a practitioner role record as not to be used because it was created in error, or otherwise no longer in active use.</t>
-  </si>
-  <si>
-    <t>This resource is generally assumed to be active if no value is provided for the active element</t>
-  </si>
-  <si>
-    <t>STF-7</t>
-  </si>
-  <si>
-    <t>.statusCode</t>
-  </si>
-  <si>
-    <t>FiveWs.status</t>
-  </si>
-  <si>
-    <t>PractitionerRole.period</t>
-  </si>
-  <si>
-    <t>The period during which the practitioner is authorized to perform in these role(s)</t>
-  </si>
-  <si>
-    <t>The period during which the person is authorized to act as a practitioner in these role(s) for the organization.</t>
-  </si>
-  <si>
-    <t>Even after the agencies is revoked, the fact that it existed must still be recorded.</t>
-  </si>
-  <si>
-    <t>PRD-8/9 / PRA-5.4</t>
-  </si>
-  <si>
-    <t>.performance[@typeCode &lt;= 'PPRF'].ActDefinitionOrEvent.effectiveTime</t>
-  </si>
-  <si>
-    <t>(ServD maps Practitioners and Organizations via another entity, so this concept is not available)</t>
-  </si>
-  <si>
-    <t>FiveWs.done[x]</t>
-  </si>
-  <si>
-    <t>PractitionerRole.practitioner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-practitioner)
-</t>
-  </si>
-  <si>
-    <t>Practitioner that is able to provide the defined services for the organization</t>
-  </si>
-  <si>
-    <t>Practitioner that is able to provide the defined services for the organization.</t>
-  </si>
-  <si>
-    <t>References SHALL be a reference to an actual FHIR resource, and SHALL be resolveable (allowing for access control, temporary unavailability, etc.). Resolution can be either by retrieval from the URL, or, where applicable by resource type, by treating an absolute reference as a canonical URL and looking it up in a local registry/repository.</t>
-  </si>
-  <si>
-    <t>.player</t>
-  </si>
-  <si>
-    <t>PractitionerRole.organization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-organization)
-</t>
-  </si>
-  <si>
-    <t>Organization where the roles are available</t>
-  </si>
-  <si>
-    <t>The organization where the Practitioner performs the roles associated.</t>
-  </si>
-  <si>
-    <t>.scoper</t>
-  </si>
-  <si>
-    <t>PractitionerRole.code</t>
-  </si>
-  <si>
     <t>The role a person plays representing an organization | Rôle (situation d'exercice) du professionnel de santé au sein de l'organisation</t>
   </si>
   <si>
@@ -1008,6 +838,9 @@
   </si>
   <si>
     <t>Not all terminology uses fit this general pattern. In some cases, models should not use CodeableConcept and use Coding directly and provide their own structure for managing text, codings, translations and the relationship between elements and pre- and post-coordination.</t>
+  </si>
+  <si>
+    <t>required</t>
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-practitioner-specialty</t>
@@ -1562,7 +1395,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN54"/>
+  <dimension ref="A1:AN46"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="46.96875" customWidth="true" bestFit="true"/>
@@ -1584,7 +1417,7 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="38.2265625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="9.953125" customWidth="true" bestFit="true"/>
     <col min="21" max="21" width="17.171875" customWidth="true" bestFit="true"/>
     <col min="22" max="22" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
@@ -1601,7 +1434,7 @@
     <col min="34" max="34" width="11.0390625" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
     <col min="37" max="37" width="85.47265625" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="102.6171875" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="78.58203125" customWidth="true" bestFit="true"/>
     <col min="39" max="39" width="194.47265625" customWidth="true" bestFit="true"/>
     <col min="40" max="40" width="36.91796875" customWidth="true" bestFit="true"/>
   </cols>
@@ -4031,23 +3864,29 @@
         <v>78</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>105</v>
+        <v>219</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>106</v>
+        <v>220</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+        <v>221</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>222</v>
+      </c>
+      <c r="O22" t="s" s="2">
+        <v>223</v>
+      </c>
       <c r="P22" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="Q22" s="2"/>
+      <c r="Q22" t="s" s="2">
+        <v>224</v>
+      </c>
       <c r="R22" t="s" s="2">
         <v>78</v>
       </c>
@@ -4091,7 +3930,7 @@
         <v>78</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>108</v>
+        <v>218</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -4100,41 +3939,41 @@
         <v>89</v>
       </c>
       <c r="AI22" t="s" s="2">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>78</v>
+        <v>225</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>109</v>
+        <v>226</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>78</v>
+        <v>227</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>78</v>
@@ -4143,21 +3982,23 @@
         <v>78</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>112</v>
+        <v>229</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>113</v>
+        <v>230</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>114</v>
+        <v>231</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="O23" s="2"/>
+        <v>232</v>
+      </c>
+      <c r="O23" t="s" s="2">
+        <v>233</v>
+      </c>
       <c r="P23" t="s" s="2">
         <v>78</v>
       </c>
@@ -4193,51 +4034,51 @@
         <v>78</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>116</v>
+        <v>78</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>117</v>
+        <v>78</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>119</v>
+        <v>228</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>120</v>
+        <v>234</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>78</v>
+        <v>235</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>103</v>
+        <v>236</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>78</v>
+        <v>237</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>78</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4254,26 +4095,24 @@
         <v>78</v>
       </c>
       <c r="I24" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="J24" t="s" s="2">
         <v>90</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>173</v>
+        <v>240</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="O24" t="s" s="2">
-        <v>224</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
         <v>78</v>
       </c>
@@ -4297,13 +4136,13 @@
         <v>78</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>225</v>
+        <v>78</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>226</v>
+        <v>78</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>227</v>
+        <v>78</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>78</v>
@@ -4321,7 +4160,7 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -4333,13 +4172,13 @@
         <v>101</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>102</v>
+        <v>244</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="AM24" t="s" s="2">
         <v>78</v>
@@ -4350,10 +4189,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4376,20 +4215,18 @@
         <v>90</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="O25" t="s" s="2">
-        <v>235</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>78</v>
       </c>
@@ -4413,13 +4250,13 @@
         <v>78</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>153</v>
+        <v>78</v>
       </c>
       <c r="Y25" t="s" s="2">
-        <v>236</v>
+        <v>78</v>
       </c>
       <c r="Z25" t="s" s="2">
-        <v>237</v>
+        <v>78</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>78</v>
@@ -4437,7 +4274,7 @@
         <v>78</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -4449,13 +4286,13 @@
         <v>101</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>102</v>
+        <v>244</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>239</v>
+        <v>78</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>229</v>
+        <v>250</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>78</v>
@@ -4466,10 +4303,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4480,7 +4317,7 @@
         <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>78</v>
@@ -4492,19 +4329,19 @@
         <v>90</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>133</v>
+        <v>252</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>78</v>
@@ -4517,7 +4354,7 @@
         <v>78</v>
       </c>
       <c r="T26" t="s" s="2">
-        <v>245</v>
+        <v>78</v>
       </c>
       <c r="U26" t="s" s="2">
         <v>78</v>
@@ -4529,13 +4366,11 @@
         <v>78</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y26" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="Y26" s="2"/>
       <c r="Z26" t="s" s="2">
-        <v>78</v>
+        <v>257</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>78</v>
@@ -4553,13 +4388,13 @@
         <v>78</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>101</v>
@@ -4568,13 +4403,13 @@
         <v>102</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="AN26" t="s" s="2">
         <v>78</v>
@@ -4582,10 +4417,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4596,7 +4431,7 @@
         <v>79</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>78</v>
@@ -4608,16 +4443,16 @@
         <v>90</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>105</v>
+        <v>252</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -4631,7 +4466,7 @@
         <v>78</v>
       </c>
       <c r="T27" t="s" s="2">
-        <v>254</v>
+        <v>78</v>
       </c>
       <c r="U27" t="s" s="2">
         <v>78</v>
@@ -4643,13 +4478,11 @@
         <v>78</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="Y27" s="2"/>
       <c r="Z27" t="s" s="2">
-        <v>78</v>
+        <v>265</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>78</v>
@@ -4667,13 +4500,13 @@
         <v>78</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>101</v>
@@ -4682,13 +4515,13 @@
         <v>102</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>78</v>
@@ -4696,10 +4529,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4710,7 +4543,7 @@
         <v>79</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>78</v>
@@ -4722,16 +4555,16 @@
         <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4781,39 +4614,39 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>265</v>
+        <v>244</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>266</v>
+        <v>78</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>78</v>
+        <v>275</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4824,7 +4657,7 @@
         <v>79</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>78</v>
@@ -4833,19 +4666,19 @@
         <v>78</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>273</v>
+        <v>243</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4895,28 +4728,28 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>275</v>
+        <v>244</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>278</v>
+        <v>78</v>
       </c>
       <c r="AN29" t="s" s="2">
         <v>78</v>
@@ -4924,10 +4757,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4938,7 +4771,7 @@
         <v>79</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>78</v>
@@ -4947,105 +4780,101 @@
         <v>78</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="M30" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="N30" s="2"/>
+      <c r="O30" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="P30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q30" s="2"/>
+      <c r="R30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE30" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF30" t="s" s="2">
         <v>282</v>
       </c>
-      <c r="N30" t="s" s="2">
-        <v>283</v>
-      </c>
-      <c r="O30" t="s" s="2">
-        <v>284</v>
-      </c>
-      <c r="P30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q30" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="R30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE30" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF30" t="s" s="2">
-        <v>279</v>
-      </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>102</v>
+        <v>287</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>78</v>
+        <v>290</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>288</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5056,7 +4885,7 @@
         <v>79</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>78</v>
@@ -5065,23 +4894,21 @@
         <v>78</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>260</v>
+        <v>292</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="O31" t="s" s="2">
-        <v>292</v>
-      </c>
+        <v>295</v>
+      </c>
+      <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>78</v>
       </c>
@@ -5129,31 +4956,31 @@
         <v>78</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>265</v>
+        <v>102</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>293</v>
+        <v>78</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>295</v>
+        <v>78</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>296</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32">
@@ -5181,20 +5008,18 @@
         <v>78</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>298</v>
+        <v>105</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>299</v>
+        <v>106</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>300</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>301</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>78</v>
@@ -5243,7 +5068,7 @@
         <v>78</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>297</v>
+        <v>108</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -5252,16 +5077,16 @@
         <v>89</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>275</v>
+        <v>78</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>302</v>
+        <v>109</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>78</v>
@@ -5272,21 +5097,21 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>78</v>
@@ -5295,19 +5120,19 @@
         <v>78</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>304</v>
+        <v>112</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>305</v>
+        <v>113</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>306</v>
+        <v>114</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>301</v>
+        <v>115</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -5345,37 +5170,37 @@
         <v>78</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>78</v>
+        <v>116</v>
       </c>
       <c r="AC33" t="s" s="2">
-        <v>78</v>
+        <v>117</v>
       </c>
       <c r="AD33" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>303</v>
+        <v>119</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>275</v>
+        <v>120</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>307</v>
+        <v>103</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>78</v>
@@ -5386,14 +5211,14 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>78</v>
+        <v>300</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5406,25 +5231,25 @@
         <v>78</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="J34" t="s" s="2">
         <v>90</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>231</v>
+        <v>112</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>311</v>
+        <v>115</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>312</v>
+        <v>207</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>78</v>
@@ -5449,11 +5274,13 @@
         <v>78</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="Y34" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y34" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z34" t="s" s="2">
-        <v>313</v>
+        <v>78</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
@@ -5471,7 +5298,7 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5483,16 +5310,16 @@
         <v>101</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>314</v>
+        <v>78</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>315</v>
+        <v>103</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>295</v>
+        <v>78</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>78</v>
@@ -5500,10 +5327,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5523,19 +5350,19 @@
         <v>78</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>231</v>
+        <v>173</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5561,11 +5388,13 @@
         <v>78</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="Y35" s="2"/>
+        <v>264</v>
+      </c>
+      <c r="Y35" t="s" s="2">
+        <v>308</v>
+      </c>
       <c r="Z35" t="s" s="2">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>78</v>
@@ -5583,7 +5412,7 @@
         <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5598,13 +5427,13 @@
         <v>102</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>321</v>
+        <v>78</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>322</v>
+        <v>296</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>323</v>
+        <v>78</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>78</v>
@@ -5612,10 +5441,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5626,7 +5455,7 @@
         <v>79</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>78</v>
@@ -5635,20 +5464,18 @@
         <v>78</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>325</v>
+        <v>219</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>301</v>
-      </c>
+        <v>312</v>
+      </c>
+      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>78</v>
@@ -5697,39 +5524,39 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>275</v>
+        <v>102</v>
       </c>
       <c r="AK36" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>328</v>
+        <v>296</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>329</v>
+        <v>78</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>330</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5740,7 +5567,7 @@
         <v>79</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>78</v>
@@ -5752,16 +5579,16 @@
         <v>78</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>332</v>
+        <v>314</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>334</v>
+        <v>316</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5811,25 +5638,25 @@
         <v>78</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>275</v>
+        <v>102</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>335</v>
+        <v>78</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>336</v>
+        <v>296</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>78</v>
@@ -5840,10 +5667,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>337</v>
+        <v>318</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>337</v>
+        <v>318</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5854,7 +5681,7 @@
         <v>79</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>78</v>
@@ -5866,18 +5693,18 @@
         <v>78</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>338</v>
+        <v>314</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>339</v>
+        <v>319</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="N38" s="2"/>
-      <c r="O38" t="s" s="2">
-        <v>341</v>
-      </c>
+        <v>320</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>78</v>
       </c>
@@ -5925,28 +5752,28 @@
         <v>78</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>337</v>
+        <v>318</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>342</v>
+        <v>102</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>343</v>
+        <v>78</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>344</v>
+        <v>296</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>345</v>
+        <v>78</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>78</v>
@@ -5954,10 +5781,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>346</v>
+        <v>321</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>346</v>
+        <v>321</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5980,17 +5807,15 @@
         <v>78</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>347</v>
+        <v>292</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>348</v>
+        <v>322</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>350</v>
-      </c>
+        <v>323</v>
+      </c>
+      <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>78</v>
@@ -6039,7 +5864,7 @@
         <v>78</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>346</v>
+        <v>321</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
@@ -6057,7 +5882,7 @@
         <v>78</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>351</v>
+        <v>296</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>78</v>
@@ -6068,10 +5893,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>352</v>
+        <v>324</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>352</v>
+        <v>324</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6180,10 +6005,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6294,14 +6119,14 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>354</v>
+        <v>326</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>354</v>
+        <v>326</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>355</v>
+        <v>300</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6323,10 +6148,10 @@
         <v>112</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>356</v>
+        <v>301</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>357</v>
+        <v>302</v>
       </c>
       <c r="N42" t="s" s="2">
         <v>115</v>
@@ -6381,7 +6206,7 @@
         <v>78</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>358</v>
+        <v>303</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>79</v>
@@ -6410,10 +6235,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>359</v>
+        <v>327</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>359</v>
+        <v>327</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6421,10 +6246,10 @@
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>78</v>
@@ -6436,16 +6261,16 @@
         <v>78</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>173</v>
+        <v>105</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>360</v>
+        <v>328</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>361</v>
+        <v>329</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>362</v>
+        <v>307</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6471,13 +6296,13 @@
         <v>78</v>
       </c>
       <c r="X43" t="s" s="2">
-        <v>225</v>
+        <v>78</v>
       </c>
       <c r="Y43" t="s" s="2">
-        <v>363</v>
+        <v>78</v>
       </c>
       <c r="Z43" t="s" s="2">
-        <v>364</v>
+        <v>78</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>78</v>
@@ -6495,13 +6320,13 @@
         <v>78</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>359</v>
+        <v>327</v>
       </c>
       <c r="AG43" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>101</v>
@@ -6513,7 +6338,7 @@
         <v>78</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>351</v>
+        <v>109</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>78</v>
@@ -6524,10 +6349,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>365</v>
+        <v>330</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>365</v>
+        <v>330</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6550,15 +6375,17 @@
         <v>78</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>280</v>
+        <v>229</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>366</v>
+        <v>331</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>367</v>
-      </c>
-      <c r="N44" s="2"/>
+        <v>332</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>232</v>
+      </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>78</v>
@@ -6607,7 +6434,7 @@
         <v>78</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>365</v>
+        <v>330</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>79</v>
@@ -6619,13 +6446,13 @@
         <v>101</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>102</v>
+        <v>234</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>78</v>
+        <v>333</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>351</v>
+        <v>296</v>
       </c>
       <c r="AM44" t="s" s="2">
         <v>78</v>
@@ -6636,10 +6463,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>368</v>
+        <v>334</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>368</v>
+        <v>334</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6662,16 +6489,16 @@
         <v>78</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>369</v>
+        <v>105</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>370</v>
+        <v>335</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>371</v>
+        <v>336</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>372</v>
+        <v>307</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -6721,7 +6548,7 @@
         <v>78</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>368</v>
+        <v>334</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
@@ -6739,7 +6566,7 @@
         <v>78</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>351</v>
+        <v>296</v>
       </c>
       <c r="AM45" t="s" s="2">
         <v>78</v>
@@ -6750,10 +6577,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>373</v>
+        <v>337</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>373</v>
+        <v>337</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6764,7 +6591,7 @@
         <v>79</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>78</v>
@@ -6776,18 +6603,20 @@
         <v>78</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>369</v>
+        <v>338</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>374</v>
+        <v>339</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>375</v>
+        <v>340</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>372</v>
-      </c>
-      <c r="O46" s="2"/>
+        <v>243</v>
+      </c>
+      <c r="O46" t="s" s="2">
+        <v>341</v>
+      </c>
       <c r="P46" t="s" s="2">
         <v>78</v>
       </c>
@@ -6835,942 +6664,30 @@
         <v>78</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>373</v>
+        <v>337</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>102</v>
+        <v>244</v>
       </c>
       <c r="AK46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="s" s="2">
-        <v>376</v>
-      </c>
-      <c r="B47" t="s" s="2">
-        <v>376</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E47" s="2"/>
-      <c r="F47" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G47" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K47" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="L47" t="s" s="2">
-        <v>377</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="N47" s="2"/>
-      <c r="O47" s="2"/>
-      <c r="P47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q47" s="2"/>
-      <c r="R47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF47" t="s" s="2">
-        <v>376</v>
-      </c>
-      <c r="AG47" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH47" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AI47" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ47" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="AK47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL47" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="AM47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN47" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="s" s="2">
-        <v>379</v>
-      </c>
-      <c r="B48" t="s" s="2">
-        <v>379</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E48" s="2"/>
-      <c r="F48" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G48" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="H48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K48" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="L48" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
-      <c r="P48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q48" s="2"/>
-      <c r="R48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF48" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="AG48" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH48" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL48" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="AM48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K49" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="O49" s="2"/>
-      <c r="P49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q49" s="2"/>
-      <c r="R49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="AG49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AI49" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ49" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="s" s="2">
-        <v>381</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>381</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G50" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I50" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="J50" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="K50" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>357</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="O50" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="P50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q50" s="2"/>
-      <c r="R50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF50" t="s" s="2">
-        <v>358</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>383</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>384</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>362</v>
-      </c>
-      <c r="O51" s="2"/>
-      <c r="P51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="AK51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="AM51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s" s="2">
-        <v>385</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>385</v>
-      </c>
-      <c r="C52" s="2"/>
-      <c r="D52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E52" s="2"/>
-      <c r="F52" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G52" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="H52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K52" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L52" t="s" s="2">
-        <v>386</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>387</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="O52" s="2"/>
-      <c r="P52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q52" s="2"/>
-      <c r="R52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF52" t="s" s="2">
-        <v>385</v>
-      </c>
-      <c r="AG52" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
-        <v>265</v>
-      </c>
-      <c r="AK52" t="s" s="2">
-        <v>388</v>
-      </c>
-      <c r="AL52" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="AM52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="D53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E53" s="2"/>
-      <c r="F53" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G53" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="H53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K53" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="L53" t="s" s="2">
-        <v>390</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>391</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>362</v>
-      </c>
-      <c r="O53" s="2"/>
-      <c r="P53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q53" s="2"/>
-      <c r="R53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF53" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ53" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="AK53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL53" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="s" s="2">
-        <v>392</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>392</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E54" s="2"/>
-      <c r="F54" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K54" t="s" s="2">
-        <v>393</v>
-      </c>
-      <c r="L54" t="s" s="2">
-        <v>394</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>395</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="O54" t="s" s="2">
-        <v>396</v>
-      </c>
-      <c r="P54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q54" s="2"/>
-      <c r="R54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF54" t="s" s="2">
-        <v>392</v>
-      </c>
-      <c r="AG54" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AI54" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AJ54" t="s" s="2">
-        <v>275</v>
-      </c>
-      <c r="AK54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL54" t="s" s="2">
-        <v>397</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN54" t="s" s="2">
         <v>78</v>
       </c>
     </row>

</xml_diff>